<commit_message>
clean up duplicate entries
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,20 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\mudathir\all\SQLSolver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B24064-FB6F-4997-BAE2-0AF7F1D13009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC348374-A5B8-4DAC-92FA-1C5BCF3FD34D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0C7876E0-0C81-4AC0-995A-5FD1555BED28}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{0C7876E0-0C81-4AC0-995A-5FD1555BED28}"/>
   </bookViews>
   <sheets>
-    <sheet name="summary" sheetId="4" r:id="rId1"/>
-    <sheet name="cvc5_bags" sheetId="3" r:id="rId2"/>
+    <sheet name="Detail2" sheetId="7" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId2"/>
+    <sheet name="Detail1" sheetId="5" r:id="rId3"/>
+    <sheet name="summary" sheetId="4" r:id="rId4"/>
+    <sheet name="cvc5_bags" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'cvc5_bags'!$A$1:$C$145</definedName>
+    <definedName name="ExternalData_1" localSheetId="4" hidden="1">'cvc5_bags'!$A$1:$C$145</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="5" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -51,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="205">
   <si>
     <t>filename</t>
   </si>
@@ -71,9 +75,6 @@
     <t>timeout</t>
   </si>
   <si>
-    <t>/</t>
-  </si>
-  <si>
     <t>Grand Total</t>
   </si>
   <si>
@@ -516,14 +517,175 @@
   </si>
   <si>
     <t>cvc5/tpc-h/query022-call-0.smt2</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Details for Count of duration</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query026-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query040-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query059-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query090-call-2.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query076-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query054-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query222-call-2.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query127-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query143-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query222-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query151-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query176-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query193-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query193-call-4.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query050-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query048-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query035-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query126-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query126-call-4.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query191-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query211-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query218-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query013-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query026-call-4.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query107-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query039-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query044-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query051-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query106-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query089-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query062-call-4.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/spark/query070-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query073-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query082-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query088-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query120-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query156-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query161-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query220-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query172-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query185-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query219-call-0.smt2</t>
+  </si>
+  <si>
+    <t>/home/mudathir/all/SQLSolver/cvc5/calcite/query207-call-0.smt2</t>
+  </si>
+  <si>
+    <t>unfold5 filename</t>
+  </si>
+  <si>
+    <t>unfold5 result</t>
+  </si>
+  <si>
+    <t>unfold5 duration</t>
+  </si>
+  <si>
+    <t>Count of unfold5 duration</t>
+  </si>
+  <si>
+    <t>cvc5 results</t>
+  </si>
+  <si>
+    <t>Details for Count of unfold5 duration - result: unsat, unfold5 result: sat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -551,12 +713,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -583,7 +746,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Mudathir Mahgoub" refreshedDate="46135.616079050924" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="144" xr:uid="{F54DABB6-C0D6-454F-9C87-A4C893E69CDA}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Mudathir Mahgoub" refreshedDate="46135.622018402777" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="144" xr:uid="{F54DABB6-C0D6-454F-9C87-A4C893E69CDA}">
   <cacheSource type="worksheet">
     <worksheetSource name="cvc5_bags"/>
   </cacheSource>
@@ -592,12 +755,13 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="result" numFmtId="0">
-      <sharedItems count="5">
+      <sharedItems count="6">
         <s v="unsat"/>
         <s v="sat"/>
         <s v="nested star"/>
         <s v="timeout"/>
-        <s v="/"/>
+        <s v="*"/>
+        <s v="/" u="1"/>
       </sharedItems>
     </cacheField>
     <cacheField name="duration" numFmtId="0">
@@ -612,6 +776,47 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Mudathir Mahgoub" refreshedDate="46135.670673958331" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="43" xr:uid="{F8EBD9F2-C276-4C11-9591-4A309E9BEB7B}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Table1"/>
+  </cacheSource>
+  <cacheFields count="6">
+    <cacheField name="filename" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="result" numFmtId="0">
+      <sharedItems count="3">
+        <s v="sat"/>
+        <s v="timeout"/>
+        <s v="unsat"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="duration" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.0278940200805664E-2" maxValue="163.07329201698303"/>
+    </cacheField>
+    <cacheField name="unfold5 filename" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="unfold5 result" numFmtId="0">
+      <sharedItems count="3">
+        <s v="sat"/>
+        <s v="timeout"/>
+        <s v="unsat"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="unfold5 duration" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.12" maxValue="112.68899999999999"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="144">
   <r>
@@ -1333,22 +1538,379 @@
     <s v="cvc5/tpc-h/query022-call-0.smt2"/>
     <x v="2"/>
     <n v="5.2724838256835938E-2"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="43">
+  <r>
+    <s v="cvc5/calcite/query026-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.25258803367614746"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query026-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.311"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query040-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.34333968162536621"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query040-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.13800000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query059-call-0.smt2"/>
+    <x v="0"/>
+    <n v="3.0347425937652588"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query059-call-0.smt2"/>
+    <x v="1"/>
+    <n v="109.306"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query090-call-2.smt2"/>
+    <x v="0"/>
+    <n v="0.1571357250213623"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query090-call-2.smt2"/>
+    <x v="1"/>
+    <n v="109.456"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query076-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.26833939552307129"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query076-call-0.smt2"/>
+    <x v="0"/>
+    <n v="1.103"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query054-call-0.smt2"/>
+    <x v="0"/>
+    <n v="1.3379096984863281E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query054-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.22700000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query222-call-2.smt2"/>
+    <x v="0"/>
+    <n v="2.4951696395874023E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query222-call-2.smt2"/>
+    <x v="0"/>
+    <n v="1.0309999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query127-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.56582832336425781"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query127-call-0.smt2"/>
+    <x v="1"/>
+    <n v="109.121"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query143-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.11222624778747559"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query143-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.76400000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query222-call-0.smt2"/>
+    <x v="0"/>
+    <n v="2.215886116027832E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query222-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.27200000000000002"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query151-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.10030984878540039"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query151-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.27400000000000002"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query176-call-0.smt2"/>
+    <x v="0"/>
+    <n v="3.0372154712677002"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query176-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.17799999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query193-call-0.smt2"/>
+    <x v="0"/>
+    <n v="1.5712976455688477E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query193-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.156"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query193-call-4.smt2"/>
+    <x v="0"/>
+    <n v="1.6048431396484375E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query193-call-4.smt2"/>
+    <x v="0"/>
+    <n v="0.156"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query050-call-0.smt2"/>
+    <x v="1"/>
+    <n v="106.58612084388733"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query050-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.35499999999999998"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query048-call-0.smt2"/>
+    <x v="1"/>
+    <n v="129.48243546485901"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query048-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.77"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query035-call-0.smt2"/>
+    <x v="1"/>
+    <n v="140.74140596389771"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query035-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.28699999999999998"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query126-call-0.smt2"/>
+    <x v="1"/>
+    <n v="114.19701457023621"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query126-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.17"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query126-call-4.smt2"/>
+    <x v="1"/>
+    <n v="109.89438438415527"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query126-call-4.smt2"/>
+    <x v="0"/>
+    <n v="0.16700000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query191-call-0.smt2"/>
+    <x v="1"/>
+    <n v="141.05722188949585"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query191-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.36799999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query211-call-0.smt2"/>
+    <x v="1"/>
+    <n v="112.00438284873962"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query211-call-0.smt2"/>
+    <x v="1"/>
+    <n v="109.593"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query218-call-0.smt2"/>
+    <x v="1"/>
+    <n v="163.07329201698303"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query218-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.17199999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query013-call-0.smt2"/>
+    <x v="2"/>
+    <n v="8.3343029022216797E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query013-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.12"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query026-call-4.smt2"/>
+    <x v="2"/>
+    <n v="0.55092430114746094"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query026-call-4.smt2"/>
+    <x v="0"/>
+    <n v="1.0680000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query107-call-0.smt2"/>
+    <x v="2"/>
+    <n v="9.3817234039306641E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query107-call-0.smt2"/>
+    <x v="1"/>
+    <n v="112.68899999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query039-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.37451529502868652"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query039-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.22900000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query044-call-0.smt2"/>
+    <x v="2"/>
+    <n v="3.067568302154541"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query044-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.35099999999999998"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query051-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.37542366981506348"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query051-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.23200000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query106-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.12161016464233398"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query106-call-0.smt2"/>
+    <x v="1"/>
+    <n v="109.739"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query089-call-0.smt2"/>
+    <x v="2"/>
+    <n v="4.8343420028686523E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query089-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.46100000000000002"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query062-call-4.smt2"/>
+    <x v="2"/>
+    <n v="2.3318290710449219E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query062-call-4.smt2"/>
+    <x v="2"/>
+    <n v="0.185"/>
+  </r>
+  <r>
+    <s v="cvc5/spark/query070-call-0.smt2"/>
+    <x v="2"/>
+    <n v="11.522721529006958"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/spark/query070-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.28599999999999998"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query073-call-0.smt2"/>
+    <x v="2"/>
+    <n v="1.0278940200805664E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query073-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.224"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query082-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.37040281295776367"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query082-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.31"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query088-call-0.smt2"/>
+    <x v="2"/>
+    <n v="1.4728784561157227E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query088-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.14499999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query120-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.77279448509216309"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query120-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.23799999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query156-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.3668510913848877"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query156-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.23200000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query161-call-0.smt2"/>
+    <x v="2"/>
+    <n v="1.052093505859375E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query161-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.19500000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query220-call-0.smt2"/>
+    <x v="2"/>
+    <n v="3.8525581359863281E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query220-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.29599999999999999"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query172-call-0.smt2"/>
+    <x v="2"/>
+    <n v="1.5880107879638672E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query172-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.183"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query185-call-0.smt2"/>
+    <x v="2"/>
+    <n v="1.0639667510986328E-2"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query185-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.189"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query219-call-0.smt2"/>
+    <x v="2"/>
+    <n v="2.885051965713501"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query219-call-0.smt2"/>
+    <x v="0"/>
+    <n v="0.23300000000000001"/>
+  </r>
+  <r>
+    <s v="cvc5/calcite/query207-call-0.smt2"/>
+    <x v="2"/>
+    <n v="0.1787714958190918"/>
+    <s v="/home/mudathir/all/SQLSolver/cvc5/calcite/query207-call-0.smt2"/>
+    <x v="1"/>
+    <n v="108.883"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8170ABBB-621D-44CF-B48A-2F3E6EE4211B}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="3">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BC36489B-C263-464C-B6E6-C1BBFB9A89C3}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="cvc5 results" colHeaderCaption="unfold5 result">
+  <location ref="A3:E8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="6">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
-      <items count="6">
+      <items count="4">
+        <item x="0"/>
         <item x="1"/>
-        <item x="4"/>
-        <item h="1" x="2"/>
-        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
         <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1357,12 +1919,76 @@
   <rowFields count="1">
     <field x="1"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="4">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="4"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of unfold5 duration" fld="5" subtotal="count" baseField="1" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8170ABBB-621D-44CF-B48A-2F3E6EE4211B}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="3">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="1"/>
+        <item m="1" x="5"/>
+        <item h="1" x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
     </i>
     <i>
       <x v="3"/>
@@ -1405,6 +2031,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5462603E-05C9-4754-B683-680F56C80E34}" name="Table3" displayName="Table3" ref="A3:F11" totalsRowShown="0">
+  <autoFilter ref="A3:F11" xr:uid="{5462603E-05C9-4754-B683-680F56C80E34}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{92D7A31D-107D-4458-9AAF-B0B3B83D0B6D}" name="filename"/>
+    <tableColumn id="2" xr3:uid="{C4B2DEB4-2ADE-45A9-BF2C-032404814976}" name="result"/>
+    <tableColumn id="3" xr3:uid="{AF8EF1BA-ADED-4CDB-A423-07AD394D5A6D}" name="duration"/>
+    <tableColumn id="4" xr3:uid="{DB238835-A1FD-492B-BD84-5140F8B9B22A}" name="unfold5 filename"/>
+    <tableColumn id="5" xr3:uid="{01C06C5C-7A5D-4B83-AEF6-523BE9A6CD8E}" name="unfold5 result"/>
+    <tableColumn id="6" xr3:uid="{9F6AD3A6-1538-4201-9D47-252580FDFAA3}" name="unfold5 duration"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CDE0F67B-F690-457B-BDBB-0572FD68EC4B}" name="Table1" displayName="Table1" ref="A3:F46" totalsRowShown="0">
+  <autoFilter ref="A3:F46" xr:uid="{CDE0F67B-F690-457B-BDBB-0572FD68EC4B}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{325CDCE2-273A-4353-838D-6559BF3A065E}" name="filename"/>
+    <tableColumn id="2" xr3:uid="{264FD2D8-0A49-4AB9-A913-B5EC81E4BE7B}" name="result"/>
+    <tableColumn id="3" xr3:uid="{076A2C9E-A0A8-43D8-BDC3-4322F8AFAE2A}" name="duration"/>
+    <tableColumn id="4" xr3:uid="{A28F7CEB-6F4D-445F-84AB-DCFD67D47783}" name="unfold5 filename"/>
+    <tableColumn id="5" xr3:uid="{6D425250-94CD-4D5C-A8EE-6CD1B76FDA12}" name="unfold5 result"/>
+    <tableColumn id="6" xr3:uid="{084F025B-3C40-4C58-AE88-AD096ECB3591}" name="unfold5 duration"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{720D9FFD-7141-4A18-BC75-C3FB38591B4D}" name="cvc5_bags" displayName="cvc5_bags" ref="A1:C145" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:C145" xr:uid="{720D9FFD-7141-4A18-BC75-C3FB38591B4D}"/>
   <tableColumns count="3">
@@ -1732,8 +2388,1228 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B725D42-FB9E-4179-8D51-4144C5305843}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="29.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="54.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E3" t="s">
+        <v>200</v>
+      </c>
+      <c r="F3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>2.885051965713501</v>
+      </c>
+      <c r="D4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>0.23300000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>0.3668510913848877</v>
+      </c>
+      <c r="D5" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>0.77279448509216309</v>
+      </c>
+      <c r="D6" t="s">
+        <v>191</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>0.23799999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>0.37040281295776367</v>
+      </c>
+      <c r="D7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>0.37542366981506348</v>
+      </c>
+      <c r="D8" t="s">
+        <v>183</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>3.067568302154541</v>
+      </c>
+      <c r="D9" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>0.35099999999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10">
+        <v>0.37451529502868652</v>
+      </c>
+      <c r="D10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>0.22900000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>0.55092430114746094</v>
+      </c>
+      <c r="D11" t="s">
+        <v>179</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>1.0680000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702A4589-5787-4EB8-B65B-5766C3565C3C}">
+  <dimension ref="A3:E8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>11</v>
+      </c>
+      <c r="C5" s="4">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4">
+        <v>8</v>
+      </c>
+      <c r="C7" s="4">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4">
+        <v>10</v>
+      </c>
+      <c r="E7" s="4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>25</v>
+      </c>
+      <c r="C8" s="4">
+        <v>7</v>
+      </c>
+      <c r="D8" s="4">
+        <v>11</v>
+      </c>
+      <c r="E8" s="4">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{653FE020-971B-49C0-9B20-434EC9EC0541}">
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="29.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="54.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E3" t="s">
+        <v>200</v>
+      </c>
+      <c r="F3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>0.25258803367614746</v>
+      </c>
+      <c r="D4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>0.311</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>0.34333968162536621</v>
+      </c>
+      <c r="D5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>0.13800000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>3.0347425937652588</v>
+      </c>
+      <c r="D6" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>109.306</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>0.1571357250213623</v>
+      </c>
+      <c r="D7" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>109.456</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>0.26833939552307129</v>
+      </c>
+      <c r="D8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>1.103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>1.3379096984863281E-2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>161</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>0.22700000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>2.4951696395874023E-2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>162</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>1.0309999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>0.56582832336425781</v>
+      </c>
+      <c r="D11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E11" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>109.121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>0.11222624778747559</v>
+      </c>
+      <c r="D12" t="s">
+        <v>164</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>0.76400000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>2.215886116027832E-2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>165</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13">
+        <v>0.27200000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>0.10030984878540039</v>
+      </c>
+      <c r="D14" t="s">
+        <v>166</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>0.27400000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>3.0372154712677002</v>
+      </c>
+      <c r="D15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15">
+        <v>0.17799999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>1.5712976455688477E-2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>0.156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>1.6048431396484375E-2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>169</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>0.156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18">
+        <v>106.58612084388733</v>
+      </c>
+      <c r="D18" t="s">
+        <v>170</v>
+      </c>
+      <c r="E18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>0.35499999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19">
+        <v>129.48243546485901</v>
+      </c>
+      <c r="D19" t="s">
+        <v>171</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20">
+        <v>140.74140596389771</v>
+      </c>
+      <c r="D20" t="s">
+        <v>172</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20">
+        <v>0.28699999999999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <v>114.19701457023621</v>
+      </c>
+      <c r="D21" t="s">
+        <v>173</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>109.89438438415527</v>
+      </c>
+      <c r="D22" t="s">
+        <v>174</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22">
+        <v>0.16700000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>141.05722188949585</v>
+      </c>
+      <c r="D23" t="s">
+        <v>175</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23">
+        <v>0.36799999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>112.00438284873962</v>
+      </c>
+      <c r="D24" t="s">
+        <v>176</v>
+      </c>
+      <c r="E24" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24">
+        <v>109.593</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" t="s">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>163.07329201698303</v>
+      </c>
+      <c r="D25" t="s">
+        <v>177</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25">
+        <v>0.17199999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26">
+        <v>8.3343029022216797E-2</v>
+      </c>
+      <c r="D26" t="s">
+        <v>178</v>
+      </c>
+      <c r="E26" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27">
+        <v>0.55092430114746094</v>
+      </c>
+      <c r="D27" t="s">
+        <v>179</v>
+      </c>
+      <c r="E27" t="s">
+        <v>3</v>
+      </c>
+      <c r="F27">
+        <v>1.0680000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28">
+        <v>9.3817234039306641E-2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>180</v>
+      </c>
+      <c r="E28" t="s">
+        <v>5</v>
+      </c>
+      <c r="F28">
+        <v>112.68899999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29">
+        <v>0.37451529502868652</v>
+      </c>
+      <c r="D29" t="s">
+        <v>181</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>0.22900000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30">
+        <v>3.067568302154541</v>
+      </c>
+      <c r="D30" t="s">
+        <v>182</v>
+      </c>
+      <c r="E30" t="s">
+        <v>3</v>
+      </c>
+      <c r="F30">
+        <v>0.35099999999999998</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31">
+        <v>0.37542366981506348</v>
+      </c>
+      <c r="D31" t="s">
+        <v>183</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32">
+        <v>0.12161016464233398</v>
+      </c>
+      <c r="D32" t="s">
+        <v>184</v>
+      </c>
+      <c r="E32" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32">
+        <v>109.739</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>67</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33">
+        <v>4.8343420028686523E-2</v>
+      </c>
+      <c r="D33" t="s">
+        <v>185</v>
+      </c>
+      <c r="E33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33">
+        <v>0.46100000000000002</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34">
+        <v>2.3318290710449219E-2</v>
+      </c>
+      <c r="D34" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34">
+        <v>0.185</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35">
+        <v>11.522721529006958</v>
+      </c>
+      <c r="D35" t="s">
+        <v>187</v>
+      </c>
+      <c r="E35" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35">
+        <v>0.28599999999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36">
+        <v>1.0278940200805664E-2</v>
+      </c>
+      <c r="D36" t="s">
+        <v>188</v>
+      </c>
+      <c r="E36" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36">
+        <v>0.224</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37">
+        <v>0.37040281295776367</v>
+      </c>
+      <c r="D37" t="s">
+        <v>189</v>
+      </c>
+      <c r="E37" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38">
+        <v>1.4728784561157227E-2</v>
+      </c>
+      <c r="D38" t="s">
+        <v>190</v>
+      </c>
+      <c r="E38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38">
+        <v>0.14499999999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39">
+        <v>0.77279448509216309</v>
+      </c>
+      <c r="D39" t="s">
+        <v>191</v>
+      </c>
+      <c r="E39" t="s">
+        <v>3</v>
+      </c>
+      <c r="F39">
+        <v>0.23799999999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40">
+        <v>0.3668510913848877</v>
+      </c>
+      <c r="D40" t="s">
+        <v>192</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3</v>
+      </c>
+      <c r="F40">
+        <v>0.23200000000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41">
+        <v>1.052093505859375E-2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>193</v>
+      </c>
+      <c r="E41" t="s">
+        <v>4</v>
+      </c>
+      <c r="F41">
+        <v>0.19500000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42">
+        <v>3.8525581359863281E-2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>194</v>
+      </c>
+      <c r="E42" t="s">
+        <v>4</v>
+      </c>
+      <c r="F42">
+        <v>0.29599999999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43">
+        <v>1.5880107879638672E-2</v>
+      </c>
+      <c r="D43" t="s">
+        <v>195</v>
+      </c>
+      <c r="E43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43">
+        <v>0.183</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>45</v>
+      </c>
+      <c r="B44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44">
+        <v>1.0639667510986328E-2</v>
+      </c>
+      <c r="D44" t="s">
+        <v>196</v>
+      </c>
+      <c r="E44" t="s">
+        <v>4</v>
+      </c>
+      <c r="F44">
+        <v>0.189</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45">
+        <v>2.885051965713501</v>
+      </c>
+      <c r="D45" t="s">
+        <v>197</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3</v>
+      </c>
+      <c r="F45">
+        <v>0.23300000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>50</v>
+      </c>
+      <c r="B46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46">
+        <v>0.1787714958190918</v>
+      </c>
+      <c r="D46" t="s">
+        <v>198</v>
+      </c>
+      <c r="E46" t="s">
+        <v>5</v>
+      </c>
+      <c r="F46">
+        <v>108.883</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DCC490D-546A-42A6-BD33-EDB317158210}">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A3:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
@@ -1742,50 +3618,42 @@
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3">
-        <v>44</v>
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1793,7 +3661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62D1584C-BA2A-418E-91DD-CA929E32E58E}">
   <dimension ref="A1:C145"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1816,7 +3684,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1827,7 +3695,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -1838,7 +3706,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -1849,10 +3717,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>3.8642406463623047E-2</v>
@@ -1860,7 +3728,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
@@ -1871,7 +3739,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
         <v>3</v>
@@ -1882,7 +3750,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
@@ -1893,7 +3761,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
@@ -1904,7 +3772,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
@@ -1915,10 +3783,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>6.2798500061035156E-2</v>
@@ -1926,7 +3794,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>3</v>
@@ -1937,10 +3805,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13">
         <v>4.7407865524291992E-2</v>
@@ -1948,10 +3816,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14">
         <v>4.4548749923706055E-2</v>
@@ -1959,7 +3827,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
@@ -1970,10 +3838,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C16">
         <v>5.1749944686889648E-2</v>
@@ -1981,7 +3849,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
@@ -1992,7 +3860,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
         <v>3</v>
@@ -2003,7 +3871,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
@@ -2014,10 +3882,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20">
         <v>5.391383171081543E-2</v>
@@ -2025,7 +3893,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
@@ -2036,10 +3904,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22">
         <v>3.6230802536010742E-2</v>
@@ -2047,10 +3915,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C23">
         <v>5.4275035858154297E-2</v>
@@ -2058,10 +3926,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
       <c r="C24">
         <v>6.916046142578125E-3</v>
@@ -2069,7 +3937,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" t="s">
         <v>4</v>
@@ -2080,7 +3948,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" t="s">
         <v>5</v>
@@ -2091,7 +3959,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
         <v>5</v>
@@ -2102,7 +3970,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" t="s">
         <v>3</v>
@@ -2113,7 +3981,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B29" t="s">
         <v>3</v>
@@ -2124,10 +3992,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30">
         <v>5.3924083709716797E-2</v>
@@ -2135,7 +4003,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B31" t="s">
         <v>3</v>
@@ -2146,7 +4014,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
@@ -2157,7 +4025,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B33" t="s">
         <v>4</v>
@@ -2168,10 +4036,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C34">
         <v>3.9625644683837891E-2</v>
@@ -2179,7 +4047,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
@@ -2190,7 +4058,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B36" t="s">
         <v>3</v>
@@ -2201,7 +4069,7 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
@@ -2212,10 +4080,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C38">
         <v>0.13793778419494629</v>
@@ -2223,7 +4091,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B39" t="s">
         <v>5</v>
@@ -2234,7 +4102,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B40" t="s">
         <v>3</v>
@@ -2245,7 +4113,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B41" t="s">
         <v>3</v>
@@ -2256,7 +4124,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
@@ -2267,7 +4135,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B43" t="s">
         <v>5</v>
@@ -2278,10 +4146,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B44" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C44">
         <v>0.15719723701477051</v>
@@ -2289,7 +4157,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B45" t="s">
         <v>5</v>
@@ -2300,7 +4168,7 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B46" t="s">
         <v>4</v>
@@ -2311,7 +4179,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B47" t="s">
         <v>4</v>
@@ -2322,7 +4190,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B48" t="s">
         <v>3</v>
@@ -2333,7 +4201,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B49" t="s">
         <v>3</v>
@@ -2344,10 +4212,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C50">
         <v>5.1884889602661133E-2</v>
@@ -2355,10 +4223,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C51">
         <v>4.5683622360229492E-2</v>
@@ -2366,7 +4234,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B52" t="s">
         <v>5</v>
@@ -2377,7 +4245,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B53" t="s">
         <v>5</v>
@@ -2388,7 +4256,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B54" t="s">
         <v>3</v>
@@ -2399,10 +4267,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B55" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C55">
         <v>2.1603503227233887</v>
@@ -2410,10 +4278,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C56">
         <v>6.6708564758300781E-2</v>
@@ -2421,10 +4289,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C57">
         <v>0.63663554191589355</v>
@@ -2432,7 +4300,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B58" t="s">
         <v>4</v>
@@ -2443,7 +4311,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
@@ -2454,7 +4322,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B60" t="s">
         <v>3</v>
@@ -2465,7 +4333,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B61" t="s">
         <v>4</v>
@@ -2476,7 +4344,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
@@ -2487,10 +4355,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C63">
         <v>5.2588939666748047E-2</v>
@@ -2498,10 +4366,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C64">
         <v>6.0362577438354492E-2</v>
@@ -2509,10 +4377,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C65">
         <v>6.1455726623535156E-2</v>
@@ -2520,10 +4388,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C66">
         <v>5.9892416000366211E-2</v>
@@ -2531,10 +4399,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C67">
         <v>6.0211420059204102E-2</v>
@@ -2542,10 +4410,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B68" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C68">
         <v>6.128692626953125E-2</v>
@@ -2553,10 +4421,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B69" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C69">
         <v>5.9460639953613281E-2</v>
@@ -2564,10 +4432,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C70">
         <v>6.4562797546386719E-2</v>
@@ -2575,10 +4443,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B71" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C71">
         <v>6.2532663345336914E-2</v>
@@ -2586,10 +4454,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B72" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C72">
         <v>5.8574914932250977E-2</v>
@@ -2597,10 +4465,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B73" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C73">
         <v>5.7337522506713867E-2</v>
@@ -2608,10 +4476,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B74" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C74">
         <v>5.7479143142700195E-2</v>
@@ -2619,10 +4487,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B75" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C75">
         <v>5.9191226959228516E-2</v>
@@ -2630,10 +4498,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B76" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C76">
         <v>5.9611320495605469E-2</v>
@@ -2641,10 +4509,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B77" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C77">
         <v>5.6119203567504883E-2</v>
@@ -2652,10 +4520,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C78">
         <v>5.6780815124511719E-2</v>
@@ -2663,10 +4531,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B79" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C79">
         <v>5.7271242141723633E-2</v>
@@ -2674,10 +4542,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B80" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C80">
         <v>5.5877447128295898E-2</v>
@@ -2685,10 +4553,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B81" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C81">
         <v>7.8125715255737305E-2</v>
@@ -2696,10 +4564,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C82">
         <v>5.9170246124267578E-2</v>
@@ -2707,10 +4575,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C83">
         <v>5.9299230575561523E-2</v>
@@ -2718,10 +4586,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C84">
         <v>5.6706428527832031E-2</v>
@@ -2729,10 +4597,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B85" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C85">
         <v>5.7913303375244141E-2</v>
@@ -2740,10 +4608,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B86" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C86">
         <v>5.6421995162963867E-2</v>
@@ -2751,10 +4619,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C87">
         <v>6.2288045883178711E-2</v>
@@ -2762,10 +4630,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B88" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C88">
         <v>5.47332763671875E-2</v>
@@ -2773,10 +4641,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B89" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C89">
         <v>5.9818029403686523E-2</v>
@@ -2784,10 +4652,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B90" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C90">
         <v>5.8639764785766602E-2</v>
@@ -2795,10 +4663,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B91" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C91">
         <v>5.7395458221435547E-2</v>
@@ -2806,10 +4674,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B92" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C92">
         <v>5.5633783340454102E-2</v>
@@ -2817,10 +4685,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B93" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C93">
         <v>6.8532943725585938E-2</v>
@@ -2828,10 +4696,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B94" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C94">
         <v>6.8268537521362305E-2</v>
@@ -2839,10 +4707,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B95" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C95">
         <v>5.5817842483520508E-2</v>
@@ -2850,10 +4718,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B96" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C96">
         <v>7.6503515243530273E-2</v>
@@ -2861,10 +4729,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B97" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C97">
         <v>5.8577060699462891E-2</v>
@@ -2872,10 +4740,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C98">
         <v>6.2987327575683594E-2</v>
@@ -2883,10 +4751,10 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B99" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C99">
         <v>5.7950496673583984E-2</v>
@@ -2894,10 +4762,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C100">
         <v>5.4963827133178711E-2</v>
@@ -2905,10 +4773,10 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B101" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C101">
         <v>6.0113906860351563E-2</v>
@@ -2916,10 +4784,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C102">
         <v>6.3482284545898438E-2</v>
@@ -2927,10 +4795,10 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B103" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C103">
         <v>6.039881706237793E-2</v>
@@ -2938,10 +4806,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C104">
         <v>6.3306093215942383E-2</v>
@@ -2949,10 +4817,10 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C105">
         <v>5.8670282363891602E-2</v>
@@ -2960,10 +4828,10 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B106" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C106">
         <v>5.6482076644897461E-2</v>
@@ -2971,10 +4839,10 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B107" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C107">
         <v>5.9742212295532227E-2</v>
@@ -2982,10 +4850,10 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B108" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C108">
         <v>5.9169530868530273E-2</v>
@@ -2993,10 +4861,10 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B109" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C109">
         <v>6.0022830963134766E-2</v>
@@ -3004,10 +4872,10 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C110">
         <v>6.2269687652587891E-2</v>
@@ -3015,10 +4883,10 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B111" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C111">
         <v>6.044459342956543E-2</v>
@@ -3026,10 +4894,10 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B112" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C112">
         <v>6.0007572174072266E-2</v>
@@ -3037,10 +4905,10 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B113" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C113">
         <v>6.2320232391357422E-2</v>
@@ -3048,10 +4916,10 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B114" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C114">
         <v>5.6116819381713867E-2</v>
@@ -3059,10 +4927,10 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B115" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C115">
         <v>5.3966522216796875E-2</v>
@@ -3070,10 +4938,10 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B116" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C116">
         <v>5.4231166839599609E-2</v>
@@ -3081,10 +4949,10 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B117" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C117">
         <v>5.4654598236083984E-2</v>
@@ -3092,10 +4960,10 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B118" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C118">
         <v>5.3322076797485352E-2</v>
@@ -3103,10 +4971,10 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C119">
         <v>5.5099964141845703E-2</v>
@@ -3114,10 +4982,10 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B120" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C120">
         <v>5.5531740188598633E-2</v>
@@ -3125,10 +4993,10 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B121" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C121">
         <v>5.3765058517456055E-2</v>
@@ -3136,10 +5004,10 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B122" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C122">
         <v>5.3495883941650391E-2</v>
@@ -3147,10 +5015,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B123" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C123">
         <v>6.4901351928710938E-2</v>
@@ -3158,10 +5026,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B124" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C124">
         <v>6.3427448272705078E-2</v>
@@ -3169,10 +5037,10 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B125" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C125">
         <v>6.6490888595581055E-2</v>
@@ -3180,10 +5048,10 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B126" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C126">
         <v>6.5603733062744141E-2</v>
@@ -3191,10 +5059,10 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B127" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C127">
         <v>6.5168380737304688E-2</v>
@@ -3202,10 +5070,10 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B128" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C128">
         <v>6.3452005386352539E-2</v>
@@ -3213,10 +5081,10 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B129" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C129">
         <v>6.3229560852050781E-2</v>
@@ -3224,10 +5092,10 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B130" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C130">
         <v>6.612396240234375E-2</v>
@@ -3235,10 +5103,10 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B131" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C131">
         <v>6.3099861145019531E-2</v>
@@ -3246,10 +5114,10 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B132" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C132">
         <v>7.3638439178466797E-2</v>
@@ -3257,10 +5125,10 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B133" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C133">
         <v>6.3541173934936523E-2</v>
@@ -3268,10 +5136,10 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B134" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C134">
         <v>6.6741466522216797E-2</v>
@@ -3279,10 +5147,10 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B135" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C135">
         <v>6.0814380645751953E-2</v>
@@ -3290,10 +5158,10 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B136" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C136">
         <v>7.2372674942016602E-2</v>
@@ -3301,10 +5169,10 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B137" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C137">
         <v>7.4596405029296875E-2</v>
@@ -3312,10 +5180,10 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B138" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C138">
         <v>7.0557594299316406E-2</v>
@@ -3323,10 +5191,10 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B139" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C139">
         <v>6.6439151763916016E-2</v>
@@ -3334,10 +5202,10 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B140" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C140">
         <v>6.3963890075683594E-2</v>
@@ -3345,10 +5213,10 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B141" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C141">
         <v>0.14806723594665527</v>
@@ -3356,10 +5224,10 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B142" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C142">
         <v>5.6180477142333984E-2</v>
@@ -3367,10 +5235,10 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B143" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C143">
         <v>6.7574262619018555E-2</v>
@@ -3378,10 +5246,10 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B144" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C144">
         <v>4.6711444854736328E-2</v>
@@ -3389,10 +5257,10 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B145" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C145">
         <v>5.2724838256835938E-2</v>

</xml_diff>